<commit_message>
chore(roadmap): remove GitHub Org Setup and VDI Tooling Setup rows, renumber
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J54"/>
+  <dimension ref="B2:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -793,17 +793,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>GitHub Org Setup</t>
+          <t>Inventory Finalization</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Provision the GitHub Enterprise Cloud org. Configure Entra SSO and SCIM. Set org-wide defaults: main as default branch, secret scanning enabled, push protection on.</t>
+          <t>Confirm the 309 active repos, agree on batch groupings, resolve the 3 collision renames, and confirm disposition of the 18 empty repos.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Platform Team</t>
+          <t>Engineer and Lead</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -823,97 +823,97 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>GitHub org live with SSO working</t>
+          <t>Finalized Repo Inventory with batch assignments</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Phase 0</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>VDI Tooling Setup</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Install embeddable Python on VDI, set up dependencies, clone the migration repo, and configure the .env file with credentials.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Script - Mirror Migration</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Build git_mirror_migrate.py to clone each repo from ADO and push it to GitHub. Includes dry-run mode, retry on failure, resume capability, and the master to main rename option.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>14 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>16 Jul 2026</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>All scripts runnable on VDI</t>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>21 Jul 2026</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>25 Jul 2026</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>git_mirror_migrate.py ready</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Phase 0</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Inventory Finalization</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Confirm the 309 active repos, agree on batch groupings, resolve the 3 collision renames, and confirm disposition of the 18 empty repos.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Engineer and Lead</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>14 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>19 Jul 2026</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Script - Topics and Teams</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Build apply_topics_teams.py to set GitHub topics and team permissions for each repo based on the workbook. Dry-run and idempotent.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>21 Jul 2026</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>25 Jul 2026</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Finalized Repo Inventory with batch assignments</t>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>apply_topics_teams.py ready</t>
         </is>
       </c>
     </row>
@@ -928,12 +928,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Script - Mirror Migration</t>
+          <t>Script - Branch Rulesets</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Build git_mirror_migrate.py to clone each repo from ADO and push it to GitHub. Includes dry-run mode, retry on failure, resume capability, and the master to main rename option.</t>
+          <t>Build apply_rulesets.py with 3 to 4 Ruleset JSON templates covering default protection, require review, file size, and comment required. Rulesets are attached by topic.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>git_mirror_migrate.py ready</t>
+          <t>apply_rulesets.py and JSON templates ready</t>
         </is>
       </c>
     </row>
@@ -973,12 +973,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Script - Topics and Teams</t>
+          <t>Script - Post-Migration Verify</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Build apply_topics_teams.py to set GitHub topics and team permissions for each repo based on the workbook. Dry-run and idempotent.</t>
+          <t>Build post_migration_verify.py to run a pass or fail check on each repo covering branch count, default branch, topics, team access, and Ruleset attachment.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -988,12 +988,12 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>apply_topics_teams.py ready</t>
+          <t>post_migration_verify.py ready</t>
         </is>
       </c>
     </row>
@@ -1018,12 +1018,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Script - Branch Rulesets</t>
+          <t>Script - CI/CD Template Applicator</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Build apply_rulesets.py with 3 to 4 Ruleset JSON templates covering default protection, require review, file size, and comment required. Rulesets are attached by topic.</t>
+          <t>Develop the standard GitHub Actions workflow YAML for identified repos. Build apply_cicd.py to push this template to each repo automatically.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1033,12 +1033,12 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>apply_rulesets.py and JSON templates ready</t>
+          <t>cicd_template.yml and apply_cicd.py ready</t>
         </is>
       </c>
     </row>
@@ -1063,22 +1063,22 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Script - Post-Migration Verify</t>
+          <t>Self-Hosted Runner Setup</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Build post_migration_verify.py to run a pass or fail check on each repo covering branch count, default branch, topics, team access, and Ruleset attachment.</t>
+          <t>Register an org-level self-hosted runner on Abank infrastructure. Validate that the runner comes online in the GitHub org and successfully picks up workflow jobs.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Engineer and Infra</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>post_migration_verify.py ready</t>
+          <t>Runner registered and online in GitHub org</t>
         </is>
       </c>
     </row>
@@ -1108,12 +1108,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Script - CI/CD Template Applicator</t>
+          <t>Script Testing on Sandbox</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Develop the standard GitHub Actions workflow YAML for identified repos. Build apply_cicd.py to push this template to each repo automatically.</t>
+          <t>Test all scripts against the zeb-ai sandbox org. Validate dry-run, retry, resume, and error handling for each script before using on Abank repos.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1138,187 +1138,187 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>cicd_template.yml and apply_cicd.py ready</t>
+          <t>All scripts passing on sandbox</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Self-Hosted Runner Setup</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Register an org-level self-hosted runner on Abank infrastructure. Validate that the runner comes online in the GitHub org and successfully picks up workflow jobs.</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Engineer and Infra</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>21 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>26 Jul 2026</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Pilot - 2 Repos</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Run the full end-to-end sequence on 2 repos: one from ScriptRefactoring and one stale single-repo project. Steps are mirror, topics, Ruleset, CI/CD, and verify. Repo owner validates the result.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>28 Jul 2026</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>29 Jul 2026</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>Runner registered and online in GitHub org</t>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>2 repos on GitHub, verify passing</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Script Testing on Sandbox</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Test all scripts against the zeb-ai sandbox org. Validate dry-run, retry, resume, and error handling for each script before using on Abank repos.</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Pilot Review and Fix</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Review what gaps were found in the pilot. Fix scripts and update the runbook. Get written sign-off to proceed to batch migration.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>26 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>28 Jul 2026</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>29 Jul 2026</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>31 Jul 2026</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>All scripts passing on sandbox</t>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Updated scripts, runbook, and sign-off</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Pilot - 2 Repos</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Run the full end-to-end sequence on 2 repos: one from ScriptRefactoring and one stale single-repo project. Steps are mirror, topics, Ruleset, CI/CD, and verify. Repo owner validates the result.</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Batch 1 - Repos 1 to 10</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Stale single-repo projects last active more than 2 years ago. Send 24 hours freeze notice, mirror, apply topics and Ruleset, verify, then archive in ADO.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>28 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>29 Jul 2026</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>31 Jul 2026</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>01 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>2 repos on GitHub, verify passing</t>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>10 repos on GitHub, ADO archived</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Pilot Review and Fix</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Review what gaps were found in the pilot. Fix scripts and update the runbook. Get written sign-off to proceed to batch migration.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Batch 2 - Repos 11 to 20</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Single-repo projects last active 1 to 2 years ago. Same freeze, mirror, topics, Ruleset, verify, archive process.</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>29 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>31 Jul 2026</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>01 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>02 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Updated scripts, runbook, and sign-off</t>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>10 repos on GitHub, ADO archived</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Batch 1 - Repos 1 to 10</t>
+          <t>Batch 3 - Repos 21 to 30</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Stale single-repo projects last active more than 2 years ago. Send 24 hours freeze notice, mirror, apply topics and Ruleset, verify, then archive in ADO.</t>
+          <t>SSIS ETL repos (5) and remaining single-repo projects. Same process as Batch 1.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1348,12 +1348,12 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>01 Aug 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -1378,12 +1378,12 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Batch 2 - Repos 11 to 20</t>
+          <t>Batch 4 - Repos 31 to 40</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Single-repo projects last active 1 to 2 years ago. Same freeze, mirror, topics, Ruleset, verify, archive process.</t>
+          <t>Non Binary repos (2) and active single-repo projects. Send 24 hours freeze notice before starting.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1393,12 +1393,12 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>01 Aug 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1423,12 +1423,12 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Batch 3 - Repos 21 to 30</t>
+          <t>Batch 5 - Repos 41 to 50</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>SSIS ETL repos (5) and remaining single-repo projects. Same process as Batch 1.</t>
+          <t>Remaining active single-repo projects. Send 24 hours freeze notice before starting.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1458,92 +1458,92 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Batch 4 - Repos 31 to 40</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Non Binary repos (2) and active single-repo projects. Send 24 hours freeze notice before starting.</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Batch 6 - Repos 51 to 60</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>ScriptRefactoring project, first 10 repos. Send 24 hours freeze notice before starting.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>03 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>04 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>07 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>08 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>10 repos on GitHub, ADO archived</t>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>10 SR repos on GitHub</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Batch 5 - Repos 41 to 50</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Remaining active single-repo projects. Send 24 hours freeze notice before starting.</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Batch 7 - Repos 61 to 70</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>ScriptRefactoring project, next 10 repos.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>04 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>05 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>08 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>09 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>10 repos on GitHub, ADO archived</t>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>10 SR repos on GitHub</t>
         </is>
       </c>
     </row>
@@ -1558,12 +1558,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Batch 6 - Repos 51 to 60</t>
+          <t>Batch 8 - Repos 71 to 80</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>ScriptRefactoring project, first 10 repos. Send 24 hours freeze notice before starting.</t>
+          <t>ScriptRefactoring project, next 10 repos.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>07 Aug 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Batch 7 - Repos 61 to 70</t>
+          <t>Batch 9 - Repos 81 to 90</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1618,12 +1618,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1648,12 +1648,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Batch 8 - Repos 71 to 80</t>
+          <t>Batch 10 - Repos 91 to 106</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>ScriptRefactoring project, next 10 repos.</t>
+          <t>ScriptRefactoring project, final 16 repos. All ScriptRefactoring repos now on GitHub.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1678,97 +1678,97 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>10 SR repos on GitHub</t>
+          <t>All 56 SR repos on GitHub</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Batch 9 - Repos 81 to 90</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring project, next 10 repos.</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Batch 11 - Repos 107 to 116</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>AB AppDev project begins. First 10 repos ordered by oldest last commit. Send 24 hours freeze notice before starting.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>10 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>11 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>14 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>15 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>10 SR repos on GitHub</t>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>10 AB AppDev repos on GitHub</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Batch 10 - Repos 91 to 106</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring project, final 16 repos. All ScriptRefactoring repos now on GitHub.</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Batch 12 - Repos 117 to 126</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>AB AppDev project, next 10 repos.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>11 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>14 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>15 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>16 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>All 56 SR repos on GitHub</t>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>10 AB AppDev repos on GitHub</t>
         </is>
       </c>
     </row>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Batch 11 - Repos 107 to 116</t>
+          <t>Batch 13 - Repos 127 to 136</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>AB AppDev project begins. First 10 repos ordered by oldest last commit. Send 24 hours freeze notice before starting.</t>
+          <t>AB AppDev project, next 10 repos.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Batch 12 - Repos 117 to 126</t>
+          <t>Batch 14 - Repos 137 to 146</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1843,12 +1843,12 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Batch 13 - Repos 127 to 136</t>
+          <t>Batch 15 - Repos 147 to 156</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Batch 14 - Repos 137 to 146</t>
+          <t>Batch 16 - Repos 157 to 166</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1933,12 +1933,12 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Batch 15 - Repos 147 to 156</t>
+          <t>Batch 17 - Repos 167 to 176</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1978,12 +1978,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Batch 16 - Repos 157 to 166</t>
+          <t>Batch 18 - Repos 177 to 186</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -2023,12 +2023,12 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Batch 17 - Repos 167 to 176</t>
+          <t>Batch 19 - Repos 187 to 196</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Batch 18 - Repos 177 to 186</t>
+          <t>Batch 20 - Repos 197 to 206</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2113,12 +2113,12 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Batch 19 - Repos 187 to 196</t>
+          <t>Batch 21 - Repos 207 to 216</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Batch 20 - Repos 197 to 206</t>
+          <t>Batch 22 - Repos 217 to 226</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2203,12 +2203,12 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Batch 21 - Repos 207 to 216</t>
+          <t>Batch 23 - Repos 227 to 236</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Batch 22 - Repos 217 to 226</t>
+          <t>Batch 24 - Repos 237 to 246</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -2293,12 +2293,12 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Batch 23 - Repos 227 to 236</t>
+          <t>Batch 25 - Repos 247 to 256</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -2338,12 +2338,12 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Batch 24 - Repos 237 to 246</t>
+          <t>Batch 26 - Repos 257 to 266</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -2383,12 +2383,12 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Batch 25 - Repos 247 to 256</t>
+          <t>Batch 27 - Repos 267 to 276</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Batch 26 - Repos 257 to 266</t>
+          <t>Batch 28 - Repos 277 to 286</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Batch 27 - Repos 267 to 276</t>
+          <t>Batch 29 - Repos 287 to 296</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -2518,12 +2518,12 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Batch 28 - Repos 277 to 286</t>
+          <t>Batch 30 - Repos 297 to 306</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2593,12 +2593,12 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Batch 29 - Repos 287 to 296</t>
+          <t>Batch 31 - Repos 307 to 309</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>AB AppDev project, next 10 repos.</t>
+          <t>AB AppDev project, final 3 repos. All 309 active repos are now on GitHub.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -2608,112 +2608,112 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>All AB AppDev repos on GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>CI/CD Repo Identification</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Identify which repos need a CI/CD pipeline. Document the pipeline type and trigger pattern for each repo before rollout begins.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Engineer and Lead</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>27 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
           <t>29 Aug 2026</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>CI/CD candidate list approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>CI/CD Pipeline Rollout</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Apply the standard GitHub Actions workflow YAML to all identified repos using apply_cicd.py. Validate that each pipeline runs successfully on the self-hosted runner.</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>27 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="I46" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>10 AB AppDev repos on GitHub</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Batch 30 - Repos 297 to 306</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev project, next 10 repos.</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>10 AB AppDev repos on GitHub</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Batch 31 - Repos 307 to 309</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev project, final 3 repos. All 309 active repos are now on GitHub.</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>All AB AppDev repos on GitHub</t>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines active, runner jobs passing</t>
         </is>
       </c>
     </row>
@@ -2728,17 +2728,17 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>CI/CD Repo Identification</t>
+          <t>Full Org Audit</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Identify which repos need a CI/CD pipeline. Document the pipeline type and trigger pattern for each repo before rollout begins.</t>
+          <t>Run post_migration_verify.py across all 309 repos. Every repo must have a project topic, correct default branch, a Ruleset applied, and team access confirmed.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Engineer and Lead</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>CI/CD candidate list approved</t>
+          <t>Audit report with all repos passing</t>
         </is>
       </c>
     </row>
@@ -2773,17 +2773,17 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>CI/CD Pipeline Rollout</t>
+          <t>Security Review</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Apply the standard GitHub Actions workflow YAML to all identified repos using apply_cicd.py. Validate that each pipeline runs successfully on the self-hosted runner.</t>
+          <t>Confirm no repos are accidentally public, secret scanning is enabled org-wide, push protection is on, and no hardcoded secrets are flagged.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>Pipelines active, runner jobs passing</t>
+          <t>Security sign-off</t>
         </is>
       </c>
     </row>
@@ -2818,127 +2818,127 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Full Org Audit</t>
+          <t>Consumer URL Updates</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Run post_migration_verify.py across all 309 repos. Every repo must have a project topic, correct default branch, a Ruleset applied, and team access confirmed.</t>
+          <t>Update any submodule references, CI clone URLs, and README badges that still point to ADO. Raise pull requests in each affected repo.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
+          <t>Team Leads</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>27 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>All consumers updated to GitHub URLs</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Phase 7</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>ADO Server Archive</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Set all ADO repos to read-only. Send communications to all teams: ADO is now archive-only and will be retained for 90 days.</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Platform Team</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>31 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>ADO read-only, comms sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Phase 7</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Runbook Handover</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Hand over the runbook to the platform team covering: how to add a new repo, apply topics, request access, change a Ruleset, and manage the runner. Includes a 1-hour walkthrough session.</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>31 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>Audit report with all repos passing</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Security Review</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Confirm no repos are accidentally public, secret scanning is enabled org-wide, push protection is on, and no hardcoded secrets are flagged.</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I50" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J50" s="5" t="inlineStr">
-        <is>
-          <t>Security sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="5" t="n">
-        <v>49</v>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Consumer URL Updates</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Update any submodule references, CI clone URLs, and README badges that still point to ADO. Raise pull requests in each affected repo.</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>Team Leads</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr">
-        <is>
-          <t>All consumers updated to GitHub URLs</t>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>Runbook delivered and session completed</t>
         </is>
       </c>
     </row>
@@ -2953,22 +2953,22 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>ADO Server Archive</t>
+          <t>ADO Decommission Planning</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Set all ADO repos to read-only. Send communications to all teams: ADO is now archive-only and will be retained for 90 days.</t>
+          <t>Plan the ADO Server decommission for 90 days after archive. Confirm the data retention policy and schedule with the Abank infrastructure team.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Platform Team</t>
+          <t>Abank Infra</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
@@ -2982,96 +2982,6 @@
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>ADO read-only, comms sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="6" t="n">
-        <v>51</v>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>Phase 7</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Runbook Handover</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>Hand over the runbook to the platform team covering: how to add a new repo, apply topics, request access, change a Ruleset, and manage the runner. Includes a 1-hour walkthrough session.</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>31 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="inlineStr">
-        <is>
-          <t>Runbook delivered and session completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Phase 7</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>ADO Decommission Planning</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>Plan the ADO Server decommission for 90 days after archive. Confirm the data retention policy and schedule with the Abank infrastructure team.</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>Abank Infra</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>31 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>31 Aug 2026</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J54" s="6" t="inlineStr">
         <is>
           <t>Decommission plan signed off</t>
         </is>
@@ -4770,7 +4680,7 @@
     </row>
     <row r="7">
       <c r="B7" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -4800,7 +4710,7 @@
     </row>
     <row r="8">
       <c r="B8" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(roadmap): remove Batch Plan and Per-Batch Process sheets
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -9,10 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions Needed" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripts to Develop" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-Batch Process" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions Needed" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripts to Develop" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2998,1250 +2996,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Batch</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Phase</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Repo Range</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Contents</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Pilot</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>2 repos</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>1 ScriptRefactoring and 1 stale single-repo</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Validation only</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>28 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>31 Jul 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Batch 1</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Repos 1-10</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Stale single-repo projects over 2 years idle</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>31 Jul 2026</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>01 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Batch 2</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Repos 11-20</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Single-repo projects 1 to 2 years idle</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>01 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>02 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Batch 3</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Repos 21-30</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>SSIS ETL (5) and single-repo projects</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Low to medium</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>02 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>03 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Batch 4</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Repos 31-40</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Non Binary (2) and active single-repo</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>03 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>04 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Batch 5</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Repos 41-50</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Remaining active single-repo projects</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>04 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>05 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Batch 6</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Repos 51-60</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring first 10</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>07 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>08 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Batch 7</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Repos 61-70</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring next 10</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>08 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>09 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Batch 8</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Repos 71-80</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring next 10</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>09 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>10 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Batch 9</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Repos 81-90</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring next 10</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>10 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>11 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Batch 10</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Repos 91-106</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>ScriptRefactoring final 16</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>SR complete</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>11 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>14 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Batch 11</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Repos 107-116</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev first 10 (oldest)</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>14 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>15 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Batch 12</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Repos 117-126</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>15 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>16 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Batch 13</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Repos 127-136</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>16 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>17 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Batch 14</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Repos 137-146</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>17 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>18 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Batch 15</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Repos 147-156</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>18 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>19 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Batch 16</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Repos 157-166</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>19 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>20 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Batch 17</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Repos 167-176</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>20 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>21 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Batch 18</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Repos 177-186</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>21 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>22 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Batch 19</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Repos 187-196</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>22 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Batch 20</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Repos 197-206</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>24 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Batch 21</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Repos 207-216</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>24 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>25 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Batch 22</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Repos 217-226</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>25 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>26 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Batch 23</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Repos 227-236</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>26 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Batch 24</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Repos 237-246</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>26 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Batch 25</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Repos 247-256</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>28 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Batch 26</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Repos 257-266</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>27 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>28 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Batch 27</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Repos 267-276</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>28 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Batch 28</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Repos 277-286</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>28 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Batch 29</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Repos 287-296</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Batch 30</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Repos 297-306</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev next 10</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Higher</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>29 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Batch 31</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Repos 307-309</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev final 3</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>All 309 migrated</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="B2:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4509,7 +3263,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4741,286 +3495,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>When</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>24h before</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Freeze Notice</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Notify repo owners via Teams or email that ADO push will be disabled in 24 hours. Share the GitHub target URL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>1h before</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Final Sync Check</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Run git fetch on the ADO repos in this batch to capture any last-minute commits before the freeze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>At cutover</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Freeze ADO</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Disable push on the ADO repos via Repos Settings. Log the exact freeze time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>At cutover</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Mirror Clone</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Run git_mirror_migrate.py in dry-run mode first. Review the output, then run live. Log any failures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>At cutover</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Apply Topics and Teams</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Run apply_topics_teams.py in dry-run mode. Review, then run live.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>At cutover</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Apply Rulesets</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Run apply_rulesets.py in dry-run mode. Review, then run live.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>At cutover</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Apply CI/CD</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Run apply_cicd.py on repos in this batch that are flagged for CI/CD. Confirm a pipeline job is queued on the runner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>1h after</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Run post_migration_verify.py. All repos in the batch must pass before the batch is marked complete.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>1h after</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Owner Validation</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Repo owner clones from GitHub, confirms branches and code look correct, and signs off.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>2h after</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Archive ADO</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Set the ADO repos to read-only. Update Status to Migrated in the Repo Inventory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>2h after</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Update Roadmap</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Mark the batch as Completed in this workbook. Commit and push to GitHub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>After</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Consumer Redirect</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Raise pull requests to update any submodule URLs, CI clone URLs, or README badges that still point to ADO.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
chore(roadmap): sync manual changes - remove Owner col, trim decisions, fix script numbering
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -674,18 +674,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J52"/>
+  <dimension ref="B2:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="49" customWidth="1" min="10" max="10"/>
+    <col width="49" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
@@ -711,25 +710,20 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>End Date</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>End Date</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>Expected Output</t>
         </is>
@@ -756,7 +750,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Project Lead</t>
+          <t>14 Jul 2026</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -766,15 +760,10 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>17 Jul 2026</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Scope sign-off and decision log</t>
         </is>
@@ -801,25 +790,20 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Engineer and Lead</t>
+          <t>15 Jul 2026</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>15 Jul 2026</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>19 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Finalized Repo Inventory with batch assignments</t>
         </is>
@@ -846,25 +830,20 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>git_mirror_migrate.py ready</t>
         </is>
@@ -891,25 +870,20 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>apply_topics_teams.py ready</t>
         </is>
@@ -936,25 +910,20 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>apply_rulesets.py and JSON templates ready</t>
         </is>
@@ -981,25 +950,20 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>post_migration_verify.py ready</t>
         </is>
@@ -1026,25 +990,20 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>cicd_template.yml and apply_cicd.py ready</t>
         </is>
@@ -1071,25 +1030,20 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Engineer and Infra</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>Runner registered and online in GitHub org</t>
         </is>
@@ -1116,25 +1070,20 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>All scripts passing on sandbox</t>
         </is>
@@ -1161,25 +1110,20 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>29 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>2 repos on GitHub, verify passing</t>
         </is>
@@ -1206,25 +1150,20 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>29 Jul 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Updated scripts, runbook, and sign-off</t>
         </is>
@@ -1251,25 +1190,20 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>01 Aug 2026</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>01 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>10 repos on GitHub, ADO archived</t>
         </is>
@@ -1296,25 +1230,20 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>01 Aug 2026</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>01 Aug 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>10 repos on GitHub, ADO archived</t>
         </is>
@@ -1341,25 +1270,20 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>10 repos on GitHub, ADO archived</t>
         </is>
@@ -1386,25 +1310,20 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>10 repos on GitHub, ADO archived</t>
         </is>
@@ -1431,25 +1350,20 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>05 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>10 repos on GitHub, ADO archived</t>
         </is>
@@ -1476,25 +1390,20 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>07 Aug 2026</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>07 Aug 2026</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>10 SR repos on GitHub</t>
         </is>
@@ -1521,25 +1430,20 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>10 SR repos on GitHub</t>
         </is>
@@ -1566,25 +1470,20 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>10 SR repos on GitHub</t>
         </is>
@@ -1611,25 +1510,20 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>10 SR repos on GitHub</t>
         </is>
@@ -1656,25 +1550,20 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>All 56 SR repos on GitHub</t>
         </is>
@@ -1701,25 +1590,20 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -1746,25 +1630,20 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -1791,25 +1670,20 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -1836,25 +1710,20 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -1881,25 +1750,20 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -1926,25 +1790,20 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -1971,25 +1830,20 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2016,25 +1870,20 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2061,25 +1910,20 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2106,25 +1950,20 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2151,25 +1990,20 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2196,25 +2030,20 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2241,25 +2070,20 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2286,25 +2110,20 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2331,25 +2150,20 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2376,25 +2190,20 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2421,25 +2230,20 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2466,25 +2270,20 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2511,25 +2310,20 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2556,25 +2350,20 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
         <is>
           <t>10 AB AppDev repos on GitHub</t>
         </is>
@@ -2601,7 +2390,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2611,15 +2400,10 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
         <is>
           <t>All AB AppDev repos on GitHub</t>
         </is>
@@ -2646,25 +2430,20 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Engineer and Lead</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>CI/CD candidate list approved</t>
         </is>
@@ -2691,25 +2470,20 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J46" s="5" t="inlineStr">
         <is>
           <t>Pipelines active, runner jobs passing</t>
         </is>
@@ -2736,25 +2510,20 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>Audit report with all repos passing</t>
         </is>
@@ -2781,25 +2550,20 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr">
         <is>
           <t>Security sign-off</t>
         </is>
@@ -2826,25 +2590,20 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Team Leads</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
         <is>
           <t>All consumers updated to GitHub URLs</t>
         </is>
@@ -2871,25 +2630,20 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>Platform Team</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="inlineStr">
         <is>
           <t>ADO read-only, comms sent</t>
         </is>
@@ -2916,25 +2670,20 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="inlineStr">
         <is>
           <t>Runbook delivered and session completed</t>
         </is>
@@ -2961,7 +2710,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Abank Infra</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -2971,15 +2720,10 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>Decommission plan signed off</t>
         </is>
@@ -2996,13 +2740,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F11"/>
+  <dimension ref="B2:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3114,22 +2858,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PR history</t>
+          <t>Self-hosted runner infrastructure</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>The git mirror approach does not carry over pull requests or PR comments. Teams lose this history unless an alternative is arranged.</t>
+          <t>What server or VM will host the org-level self-hosted runner, and who is responsible for maintaining it?</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Project Lead and Management</t>
+          <t>Abank Infra</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Accept the loss and keep ADO read-only for 90 days as a reference (recommended) or engage GitHub Professional Services for a custom exporter</t>
+          <t>Dedicated VM (recommended) or reuse an existing build server</t>
         </is>
       </c>
     </row>
@@ -3139,120 +2883,20 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>325 unprotected repos</t>
+          <t>ADO archive retention period</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Only 2 repos had branch policies in ADO. Should we apply Rulesets to all repos on GitHub to establish a consistent baseline?</t>
+          <t>How long should ADO repos remain read-only after cutover before the server is decommissioned?</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Project Lead</t>
+          <t>Abank IT Management</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Apply a default protection Ruleset org-wide (recommended) or migrate with no branch protection</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>GitHub org name</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>What is the GitHub Enterprise Cloud org name? It should align with Abank branding.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Abank IT Management</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>To be confirmed by Abank</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>CI/CD repos in scope</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Which repos need a CI/CD pipeline configured? This list must be agreed before Phase 6 begins.</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Project Lead and Dev Leads</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Identify by tech stack such as dotnet, python, or node, combined with deployment target</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Self-hosted runner infrastructure</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>What server or VM will host the org-level self-hosted runner, and who is responsible for maintaining it?</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Abank Infra</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Dedicated VM (recommended) or reuse an existing build server</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>ADO archive retention period</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>How long should ADO repos remain read-only after cutover before the server is decommissioned?</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Abank IT Management</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>90 days (recommended), 6 months, or permanent</t>
         </is>
@@ -3434,7 +3078,7 @@
     </row>
     <row r="7">
       <c r="B7" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -3464,7 +3108,7 @@
     </row>
     <row r="8">
       <c r="B8" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(roadmap): remove date gap between Phase 0 and Phase 1, flow continuously to 26 Aug
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>16 Jul 2026</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>20 Jul 2026</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -870,12 +870,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>16 Jul 2026</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>20 Jul 2026</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>16 Jul 2026</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>20 Jul 2026</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -950,12 +950,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1030,12 +1030,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
+          <t>16 Jul 2026</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
           <t>21 Jul 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>29 Jul 2026</t>
+          <t>24 Jul 2026</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>29 Jul 2026</t>
+          <t>24 Jul 2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>01 Aug 2026</t>
+          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>01 Aug 2026</t>
+          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>30 Jul 2026</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>30 Jul 2026</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>05 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>07 Aug 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1470,12 +1470,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>13 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1750,12 +1750,12 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>13 Aug 2026</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2190,12 +2190,12 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2230,12 +2230,12 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2310,12 +2310,12 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -2550,12 +2550,12 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -2590,12 +2590,12 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -2630,12 +2630,12 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
@@ -2670,12 +2670,12 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
@@ -2710,12 +2710,12 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">

</xml_diff>

<commit_message>
fix(roadmap): skip weekends in date calculation, end date 11 Sep 2026
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>11 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Approx. 7 weeks</t>
+          <t>Approx. 9 weeks (weekends excluded)</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>20 Jul 2026</t>
+          <t>22 Jul 2026</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>20 Jul 2026</t>
+          <t>22 Jul 2026</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>20 Jul 2026</t>
+          <t>22 Jul 2026</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -950,12 +950,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>18 Jul 2026</t>
+          <t>20 Jul 2026</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>18 Jul 2026</t>
+          <t>20 Jul 2026</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>24 Jul 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>24 Jul 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>30 Jul 2026</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>26 Jul 2026</t>
+          <t>30 Jul 2026</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>27 Jul 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>27 Jul 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>29 Jul 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>29 Jul 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>30 Jul 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>30 Jul 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1470,12 +1470,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>05 Aug 2026</t>
+          <t>13 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>05 Aug 2026</t>
+          <t>13 Aug 2026</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>06 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>06 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>09 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>12 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>12 Aug 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>13 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1750,12 +1750,12 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>13 Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>15 Aug 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>16 Aug 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>01 Sep 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>01 Sep 2026</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>02 Sep 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>02 Sep 2026</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>03 Sep 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>03 Sep 2026</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>04 Sep 2026</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>04 Sep 2026</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>04 Sep 2026</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2190,12 +2190,12 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2230,12 +2230,12 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2310,12 +2310,12 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -2550,12 +2550,12 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>09 Sep 2026</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -2590,12 +2590,12 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>22 Aug 2026</t>
+          <t>07 Sep 2026</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -2630,12 +2630,12 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>11 Sep 2026</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
@@ -2670,12 +2670,12 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>10 Sep 2026</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>11 Sep 2026</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
@@ -2710,12 +2710,12 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>11 Sep 2026</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>11 Sep 2026</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">

</xml_diff>

<commit_message>
fix(roadmap): scale dates to end exactly 31 Aug, weekends skipped
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>11 Sep 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Approx. 9 weeks (weekends excluded)</t>
+          <t>Approx. 7 weeks (weekends excluded)</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>22 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>22 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>22 Jul 2026</t>
+          <t>21 Jul 2026</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -950,12 +950,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>20 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>22 Jul 2026</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>20 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>22 Jul 2026</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>23 Jul 2026</t>
+          <t>22 Jul 2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
+          <t>22 Jul 2026</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
           <t>23 Jul 2026</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>27 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>24 Jul 2026</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>24 Jul 2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>30 Jul 2026</t>
+          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>30 Jul 2026</t>
+          <t>27 Jul 2026</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>31 Jul 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>30 Jul 2026</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>30 Jul 2026</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>05 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>05 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>06 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>12 Aug 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1470,12 +1470,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>12 Aug 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>13 Aug 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>13 Aug 2026</t>
+          <t>06 Aug 2026</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>07 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>14 Aug 2026</t>
+          <t>07 Aug 2026</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>19 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>20 Aug 2026</t>
+          <t>12 Aug 2026</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>13 Aug 2026</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>21 Aug 2026</t>
+          <t>13 Aug 2026</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>24 Aug 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1750,12 +1750,12 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>26 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>27 Aug 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>28 Aug 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>02 Sep 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>02 Sep 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>03 Sep 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>03 Sep 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>04 Sep 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>04 Sep 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>04 Sep 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2190,12 +2190,12 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2230,12 +2230,12 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2310,12 +2310,12 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -2550,12 +2550,12 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -2590,12 +2590,12 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>07 Sep 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -2630,12 +2630,12 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>11 Sep 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
@@ -2670,12 +2670,12 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>10 Sep 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>11 Sep 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
@@ -2710,12 +2710,12 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>11 Sep 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>11 Sep 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">

</xml_diff>

<commit_message>
chore(roadmap): sync manual changes - remove Client row, trim phases/duration, mark row 1 Completed
</commit_message>
<xml_diff>
--- a/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Abank Document/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C15"/>
+  <dimension ref="B2:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -510,156 +510,142 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Amalgamated Bank (Abank)</t>
+          <t>Azure DevOps Server on-prem (abdevopsdev, API 5.1)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps Server on-prem (abdevopsdev, API 5.1)</t>
+          <t>GitHub Enterprise Cloud (Standard)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Total Repos</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>GitHub Enterprise Cloud (Standard)</t>
+          <t>327</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Total Repos</t>
+          <t>Active Repos to Migrate</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>327</t>
+          <t>309 (18 empty repos excluded, confirmed skip)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Active Repos to Migrate</t>
+          <t>ADO Projects</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>309 (18 empty repos excluded, confirmed skip)</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ADO Projects</t>
+          <t>Migration Approach</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>git push mirror from VDI. GEI not supported for on-prem ADO Server.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Migration Approach</t>
+          <t>Batch Size</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>git push mirror from VDI. GEI not supported for on-prem ADO Server.</t>
+          <t>10 repos per batch</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Batch Size</t>
+          <t>Total Batches</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>10 repos per batch</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Total Batches</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+          <t>Total Phases</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Total Phases</t>
+          <t>Planned Start</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>8 (Phase 0 through Phase 7)</t>
+          <t>14 Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Planned Start</t>
+          <t>Planned End</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Planned End</t>
+          <t>Total Duration</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>31 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Total Duration</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Approx. 7 weeks (weekends excluded)</t>
+          <t>Approx</t>
         </is>
       </c>
     </row>
@@ -760,7 +746,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">

</xml_diff>